<commit_message>
fix bwUpper/bwCatString handling and update import format templates; closes #1324
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/records/importFormatRecords.xlsx
+++ b/owlcms/src/main/resources/templates/records/importFormatRecords.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\templates\records\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\git\owlcms_v23\owlcms\src\main\resources\templates\records\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{801D8CA5-7EB0-4DD4-9B64-F9EAFDE9EEF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8D89E9C-54AA-4A5B-B9B4-B8F05CF2B340}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2370" yWindow="1065" windowWidth="22485" windowHeight="13980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Records" sheetId="1" r:id="rId1"/>
@@ -84,8 +84,7 @@
           <t xml:space="preserve">
 for non-heavyweight category use a number
 45 59 55 64 ...
-for heavyweight category use &gt; followed by number
-&gt;81 &gt;87 &gt;102 &gt;109 </t>
+for heavyweight category use 999</t>
         </r>
       </text>
     </comment>
@@ -1229,8 +1228,8 @@
       <c r="O29" s="7"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H1 G1:G1048576 H3:H1048576" xr:uid="{53FB7450-D8BD-4FB4-A0E8-29CC05EF8875}">
+  <dataValidations count="3">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G1:G1048576" xr:uid="{53FB7450-D8BD-4FB4-A0E8-29CC05EF8875}">
       <formula1>0</formula1>
       <formula2>250</formula2>
     </dataValidation>
@@ -1238,6 +1237,10 @@
       <formula1>0</formula1>
       <formula2>120</formula2>
     </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H1:H1048576" xr:uid="{905FFAC0-C9A6-475E-9DE4-6B5BF21663BF}">
+      <formula1>0</formula1>
+      <formula2>999</formula2>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>